<commit_message>
COL 18 - Ajustes hoja de entrada de excel con valores reales del sistema
Térmica, hidráulica, solar, y demanda
</commit_message>
<xml_diff>
--- a/01_Data/02_Processed/Datos_hojas_excel_COL/18_nodos/03_Hidraulicos/hidraulicos_trazabilidad.xlsx
+++ b/01_Data/02_Processed/Datos_hojas_excel_COL/18_nodos/03_Hidraulicos/hidraulicos_trazabilidad.xlsx
@@ -759,7 +759,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PORCE 3</t>
+          <t>PORCE III</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -891,7 +891,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PORCE 2</t>
+          <t>PORCE II</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1023,7 +1023,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ALTOANCHICAYA</t>
+          <t>ALTO ANCHICAYA</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2087,7 +2087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2870,17 +2870,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>costo (7 registros pendientes)</t>
+          <t>costo (plantas en cadena)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PrecOferDesp_Jul26.xlsx</t>
+          <t>PrecOferDesp_Jul26.xlsx + PARATEC_Chidraulicas.xlsx</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>01_SERIE</t>
+          <t>01_SERIE y Cadenahidráulica</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SIN ASIGNAR. Alto Anchicaya, Bajo Anchicaya, Troneras, Guadalupe III, Guadalupe IV, La Guaca y Paraiso tienen codigo vacio en PARATEC. Los codigos huerfanos ALBG, GTRG y PGUG encajarian con los recursos de despacho Alban, Guatron y Pagua, pero el emparejamiento no se hace automaticamente</t>
+          <t>El precio de oferta se publica al nivel del RECURSO DE DESPACHO, que agrupa varias plantas de una misma cadena; PARATEC deja vacio el codigo de la planta individual. Asignacion: ALBG -&gt; Alto Anchicaya + Bajo Anchicaya (cadena ALBAN, 427 MW, factor 4,0997); GTRG -&gt; Guadalupe III + Guadalupe IV + Troneras (GUATRON, 512 MW, 8,9291); PGUG -&gt; La Guaca + Paraiso (PAGUA, 600 MW, 16,0307). Verificado: la capacidad y el factor de cada cadena son la suma de los de sus plantas</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2905,12 +2905,106 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>requiere decision del usuario</t>
+          <t>PARATEC_Chidraulicas, composicion explicita</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>HALLAZGO: separador de miles en ITUANGO</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PARATEC_Detalle_Embalse.xlsx</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Información_Técnica</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>[5] y [6]</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Las celdas dicen '1.299' y '1.431'. El punto de PARATEC separa MILES: Vmin = 1 299 Mm3 y Vmax = 1 431 Mm3. Tres comprobaciones independientes: (a) 1431 - 1299 = 132 = volumen util publicado, y es el UNICO de los 29 que falla el test Vmax - Vmin = Vutil, con desfase exacto x1000; (b) la columna en GWh da 714,64 - 648,72 = 65,92, consistente; (c) CapaUtilDiarMasa de XM da 132 000 000 m3 = 132,00 Mm3, identico al util de PARATEC. NO es un problema de embalse agregado</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Mm3</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Mm3</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>NO - correccion de lectura</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>PARATEC + XM, verificacion cruzada</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>HALLAZGO: la discrepancia de agregacion XM-PARATEC no existia</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>VoluUtil/CapaUtilDiarMasa + PARATEC_Detalle_Embalse</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>La justificacion previa del metodo del porcentaje de llenado era que en tres embalses el volumen util de XM excedia el maximo tecnico de PARATEC por diferencias de agregacion entre fuentes. Con el Vmax correcto (columna [6], no la que se venia usando) las dos fuentes concuerdan dentro del 2 % en LOS 20 embalses con dinamica. La discrepancia era un artefacto de la columna equivocada. El metodo del porcentaje sigue siendo preferible por ser adimensional, pero su justificacion debe reescribirse</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>NO - correccion</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>ver hoja Comparativo_XM_PARATEC</t>
         </is>
       </c>
     </row>
@@ -7840,7 +7934,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PORCE 3</t>
+          <t>PORCE III</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -7954,7 +8048,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PORCE 2</t>
+          <t>PORCE II</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -8068,7 +8162,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ALTOANCHICAYA</t>
+          <t>ALTO ANCHICAYA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -9054,17 +9148,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>28 de 35 con costo</t>
+          <t>35 de 35 con costo</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>FALLA</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>PENDIENTE DE DECISION: ALTOANCHICAYA; TRONERAS; LA GUACA; PARAISO; GUADALUPE III; GUADALUPE IV; BAJO ANCHICAYA. Sus unidades tienen codigo vacio en PARATEC porque el codigo de oferta de XM esta al nivel del RECURSO DE DESPACHO, que agrupa varias plantas. En PrecOferDesp quedan huerfanos ALBG (285,98 USD/MWh), GTRG (193,23) y PGUG (147,63), que corresponderian a Alban, Guatron y Pagua. NO se asignan por similitud: requiere decision del usuario.</t>
+          <t>los 7 sin codigo propio se resuelven por su recurso de despacho: ALBG (Alban), GTRG (Guatron) y PGUG (Pagua), composicion verificada en PARATEC_Chidraulicas</t>
         </is>
       </c>
     </row>
@@ -9076,15 +9170,19 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>20 de 20 con lat/lon</t>
+          <t>17 de 20 con lat/lon</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PASA</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>FALLA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PORCE III; PORCE II; ALTO ANCHICAYA</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9557,7 +9655,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PORCE 3</t>
+          <t>PORCE III</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -9603,12 +9701,6 @@
           <t>PORCE III</t>
         </is>
       </c>
-      <c r="O11" t="n">
-        <v>6.9391</v>
-      </c>
-      <c r="P11" t="n">
-        <v>-75.13930000000001</v>
-      </c>
       <c r="Q11" t="inlineStr">
         <is>
           <t>con dinamica</t>
@@ -9740,7 +9832,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PORCE 2</t>
+          <t>PORCE II</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -9786,12 +9878,6 @@
           <t>PORCE II</t>
         </is>
       </c>
-      <c r="O14" t="n">
-        <v>6.798867</v>
-      </c>
-      <c r="P14" t="n">
-        <v>-75.144936</v>
-      </c>
       <c r="Q14" t="inlineStr">
         <is>
           <t>con dinamica</t>
@@ -9923,7 +10009,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ALTOANCHICAYA</t>
+          <t>ALTO ANCHICAYA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -9958,6 +10044,9 @@
       <c r="K17" t="n">
         <v>100</v>
       </c>
+      <c r="L17" t="n">
+        <v>285.9797320747624</v>
+      </c>
       <c r="M17" t="n">
         <v>90</v>
       </c>
@@ -9966,12 +10055,6 @@
           <t>ALTO ANCHICAYA</t>
         </is>
       </c>
-      <c r="O17" t="n">
-        <v>3.320507</v>
-      </c>
-      <c r="P17" t="n">
-        <v>-76.521748</v>
-      </c>
       <c r="Q17" t="inlineStr">
         <is>
           <t>con dinamica</t>
@@ -10443,6 +10526,9 @@
       <c r="K25" t="n">
         <v>100</v>
       </c>
+      <c r="L25" t="n">
+        <v>193.231956626172</v>
+      </c>
       <c r="M25" t="n">
         <v>1</v>
       </c>
@@ -10501,6 +10587,9 @@
       <c r="K26" t="n">
         <v>0</v>
       </c>
+      <c r="L26" t="n">
+        <v>147.6295237917784</v>
+      </c>
       <c r="M26" t="n">
         <v>120</v>
       </c>
@@ -10553,6 +10642,9 @@
       <c r="K27" t="n">
         <v>0</v>
       </c>
+      <c r="L27" t="n">
+        <v>147.6295237917784</v>
+      </c>
       <c r="M27" t="n">
         <v>102</v>
       </c>
@@ -10605,6 +10697,9 @@
       <c r="K28" t="n">
         <v>0</v>
       </c>
+      <c r="L28" t="n">
+        <v>193.2319566261719</v>
+      </c>
       <c r="M28" t="n">
         <v>0</v>
       </c>
@@ -10657,6 +10752,9 @@
       <c r="K29" t="n">
         <v>0</v>
       </c>
+      <c r="L29" t="n">
+        <v>193.231956626172</v>
+      </c>
       <c r="M29" t="n">
         <v>105</v>
       </c>
@@ -10928,6 +11026,9 @@
       </c>
       <c r="K34" t="n">
         <v>0</v>
+      </c>
+      <c r="L34" t="n">
+        <v>285.9797320747624</v>
       </c>
       <c r="M34" t="n">
         <v>8</v>

</xml_diff>